<commit_message>
update all code, added new computation code to compare REM vs Awake facial movements
</commit_message>
<xml_diff>
--- a/nightmareCode/comparisonPlotPaths/SGNM008_First15Minutes.xlsx
+++ b/nightmareCode/comparisonPlotPaths/SGNM008_First15Minutes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\SGNMData\comparisonPlotPaths\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\csg178\Documents\MATLAB\Workspace\DrewLab\nightmareCode\comparisonPlotPaths\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4994FFFA-1407-4BD4-BEB8-DB8480147E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB18986-8EED-452E-B79D-535B827FF66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32310" yWindow="1965" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,37 +27,37 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
-    <t>H:\SGNMData\260128\260128_13_52_3828.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260129\260129_13_29_5429.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260130\260130_11_36_3430.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260211\260211_15_14_1811.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260226\260226_11_10_4326.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260227\260227_09_39_0127.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260302\260302_11_55_2302.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260303\260303_11_19_4803.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260306\260306_12_53_4306.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260309\260309_11_26_2109.tdms</t>
-  </si>
-  <si>
-    <t>H:\SGNMData\260310\260310_11_19_1810.tdms</t>
+    <t>D:\SGNMData\260128\260128_13_52_3828.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260129\260129_13_29_5429.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260130\260130_11_36_3430.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260211\260211_15_14_1811.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260226\260226_11_10_4326.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260227\260227_09_39_0127.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260302\260302_11_55_2302.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260303\260303_11_19_4803.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260306\260306_12_53_4306.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260309\260309_11_26_2109.tdms</t>
+  </si>
+  <si>
+    <t>D:\SGNMData\260310\260310_11_19_1810.tdms</t>
   </si>
 </sst>
 </file>

</xml_diff>